<commit_message>
Update Mapping en definitie BRO SAD.xlsx
</commit_message>
<xml_diff>
--- a/BROMappings/Mapping en definitie BRO SAD.xlsx
+++ b/BROMappings/Mapping en definitie BRO SAD.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3hydro-my.sharepoint.com/personal/jos_von_asmuth_3hydro_nl/Documents/MATLAB/Menyanthes/Meny_OS/trunk/BronDatamodel/BROMappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="756" documentId="13_ncr:1_{DFE48FA1-484F-4F3E-BCD5-80D38728AFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01F3F857-7ED8-40D9-B054-81387FD3356C}"/>
+  <xr:revisionPtr revIDLastSave="767" documentId="13_ncr:1_{DFE48FA1-484F-4F3E-BCD5-80D38728AFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67174868-FB7F-42D5-8A53-EA444CF97B03}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="230">
   <si>
     <t>Registratieobject</t>
   </si>
@@ -706,6 +706,18 @@
   </si>
   <si>
     <t>EndDepth</t>
+  </si>
+  <si>
+    <t>[ParameterID]</t>
+  </si>
+  <si>
+    <t>[ConditionID]</t>
+  </si>
+  <si>
+    <t>soilSampleAnalysis</t>
+  </si>
+  <si>
+    <t>Grondmonsteranalyse</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1132,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T270"/>
+  <dimension ref="A1:T272"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -2204,13 +2216,16 @@
         <v>173</v>
       </c>
       <c r="E23" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G23" t="s">
-        <v>175</v>
+        <v>51</v>
+      </c>
+      <c r="H23" t="s">
+        <v>37</v>
       </c>
       <c r="J23"/>
       <c r="K23"/>
@@ -2219,13 +2234,13 @@
         <v>94</v>
       </c>
       <c r="P23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q23" t="s">
-        <v>170</v>
-      </c>
-      <c r="R23" s="15" t="s">
-        <v>53</v>
+        <v>169</v>
+      </c>
+      <c r="R23" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -2240,13 +2255,13 @@
         <v>173</v>
       </c>
       <c r="E24" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F24" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G24" t="s">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="J24"/>
       <c r="K24"/>
@@ -2255,13 +2270,13 @@
         <v>94</v>
       </c>
       <c r="P24" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="Q24" t="s">
-        <v>177</v>
-      </c>
-      <c r="R24" t="s">
-        <v>50</v>
+        <v>170</v>
+      </c>
+      <c r="R24" s="15" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -2270,33 +2285,34 @@
       </c>
       <c r="B25"/>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>171</v>
+      </c>
+      <c r="D25" t="s">
+        <v>173</v>
       </c>
       <c r="E25" t="s">
-        <v>87</v>
+        <v>176</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>176</v>
       </c>
       <c r="G25" t="s">
-        <v>89</v>
-      </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="N25"/>
       <c r="O25" t="s">
         <v>94</v>
       </c>
       <c r="P25" t="s">
-        <v>87</v>
+        <v>177</v>
       </c>
       <c r="Q25" t="s">
-        <v>87</v>
+        <v>177</v>
       </c>
       <c r="R25" t="s">
-        <v>89</v>
-      </c>
-      <c r="S25" t="s">
-        <v>78</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -2308,10 +2324,10 @@
         <v>105</v>
       </c>
       <c r="E26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G26" t="s">
         <v>89</v>
@@ -2322,10 +2338,10 @@
         <v>94</v>
       </c>
       <c r="P26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="Q26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="R26" t="s">
         <v>89</v>
@@ -2340,34 +2356,33 @@
       </c>
       <c r="B27"/>
       <c r="C27" t="s">
-        <v>104</v>
-      </c>
-      <c r="D27" t="s">
-        <v>142</v>
+        <v>105</v>
       </c>
       <c r="E27" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="F27" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="G27" t="s">
-        <v>138</v>
-      </c>
-      <c r="J27"/>
-      <c r="K27"/>
-      <c r="N27"/>
+        <v>89</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
       <c r="O27" t="s">
         <v>94</v>
       </c>
       <c r="P27" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="Q27" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="R27" t="s">
-        <v>138</v>
+        <v>89</v>
+      </c>
+      <c r="S27" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -2382,13 +2397,13 @@
         <v>142</v>
       </c>
       <c r="E28" t="s">
-        <v>162</v>
+        <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>163</v>
+        <v>123</v>
       </c>
       <c r="G28" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
       <c r="J28"/>
       <c r="K28"/>
@@ -2397,13 +2412,13 @@
         <v>94</v>
       </c>
       <c r="P28" t="s">
-        <v>161</v>
+        <v>103</v>
       </c>
       <c r="Q28" t="s">
-        <v>161</v>
+        <v>103</v>
       </c>
       <c r="R28" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
@@ -2412,19 +2427,19 @@
       </c>
       <c r="B29"/>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>104</v>
+      </c>
+      <c r="D29" t="s">
+        <v>142</v>
       </c>
       <c r="E29" t="s">
-        <v>107</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>121</v>
+        <v>162</v>
+      </c>
+      <c r="F29" t="s">
+        <v>163</v>
       </c>
       <c r="G29" t="s">
-        <v>175</v>
-      </c>
-      <c r="H29" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="J29"/>
       <c r="K29"/>
@@ -2433,13 +2448,13 @@
         <v>94</v>
       </c>
       <c r="P29" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="Q29" t="s">
-        <v>92</v>
-      </c>
-      <c r="R29" s="15" t="s">
-        <v>53</v>
+        <v>161</v>
+      </c>
+      <c r="R29" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
@@ -2451,31 +2466,31 @@
         <v>106</v>
       </c>
       <c r="E30" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" t="s">
-        <v>118</v>
+        <v>107</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>121</v>
       </c>
       <c r="G30" t="s">
-        <v>138</v>
+        <v>175</v>
+      </c>
+      <c r="H30" t="s">
+        <v>39</v>
       </c>
       <c r="J30"/>
       <c r="K30"/>
       <c r="N30"/>
       <c r="O30" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="P30" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="Q30" t="s">
-        <v>85</v>
-      </c>
-      <c r="R30" t="s">
-        <v>138</v>
-      </c>
-      <c r="S30" t="s">
-        <v>86</v>
+        <v>92</v>
+      </c>
+      <c r="R30" s="15" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -2487,10 +2502,10 @@
         <v>106</v>
       </c>
       <c r="E31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G31" t="s">
         <v>138</v>
@@ -2520,34 +2535,34 @@
       </c>
       <c r="B32"/>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>106</v>
       </c>
       <c r="E32" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G32" t="s">
-        <v>50</v>
-      </c>
-      <c r="H32" t="s">
-        <v>38</v>
+        <v>138</v>
       </c>
       <c r="J32"/>
       <c r="K32"/>
       <c r="N32"/>
       <c r="O32" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="P32" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="Q32" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="R32" t="s">
-        <v>50</v>
+        <v>138</v>
+      </c>
+      <c r="S32" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
@@ -2559,10 +2574,10 @@
         <v>216</v>
       </c>
       <c r="E33" t="s">
-        <v>213</v>
+        <v>99</v>
       </c>
       <c r="F33" t="s">
-        <v>214</v>
+        <v>120</v>
       </c>
       <c r="G33" t="s">
         <v>50</v>
@@ -2577,29 +2592,28 @@
         <v>94</v>
       </c>
       <c r="P33" t="s">
-        <v>212</v>
+        <v>111</v>
       </c>
       <c r="Q33" t="s">
-        <v>212</v>
+        <v>111</v>
       </c>
       <c r="R33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>159</v>
       </c>
       <c r="B34"/>
       <c r="C34" t="s">
-        <v>106</v>
-      </c>
-      <c r="D34"/>
+        <v>216</v>
+      </c>
       <c r="E34" t="s">
-        <v>97</v>
+        <v>213</v>
       </c>
       <c r="F34" t="s">
-        <v>122</v>
+        <v>214</v>
       </c>
       <c r="G34" t="s">
         <v>50</v>
@@ -2607,20 +2621,23 @@
       <c r="H34" t="s">
         <v>38</v>
       </c>
+      <c r="J34"/>
+      <c r="K34"/>
+      <c r="N34"/>
       <c r="O34" t="s">
         <v>94</v>
       </c>
       <c r="P34" t="s">
-        <v>109</v>
+        <v>212</v>
       </c>
       <c r="Q34" t="s">
-        <v>109</v>
+        <v>212</v>
       </c>
       <c r="R34" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>159</v>
       </c>
@@ -2628,11 +2645,12 @@
       <c r="C35" t="s">
         <v>106</v>
       </c>
+      <c r="D35"/>
       <c r="E35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F35" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G35" t="s">
         <v>50</v>
@@ -2640,17 +2658,14 @@
       <c r="H35" t="s">
         <v>38</v>
       </c>
-      <c r="J35"/>
-      <c r="K35"/>
-      <c r="N35"/>
       <c r="O35" t="s">
         <v>94</v>
       </c>
       <c r="P35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="R35" t="s">
         <v>50</v>
@@ -2658,84 +2673,87 @@
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>159</v>
       </c>
       <c r="B36"/>
       <c r="C36" t="s">
-        <v>69</v>
-      </c>
-      <c r="D36" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="E36" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="F36" t="s">
-        <v>69</v>
+        <v>128</v>
       </c>
       <c r="G36" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>70</v>
-      </c>
-      <c r="J36" t="s">
-        <v>70</v>
-      </c>
-      <c r="K36" t="s">
-        <v>70</v>
-      </c>
-      <c r="L36" t="s">
-        <v>70</v>
-      </c>
-      <c r="M36" t="s">
-        <v>70</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="J36"/>
+      <c r="K36"/>
       <c r="N36"/>
       <c r="O36" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="P36" t="s">
-        <v>178</v>
+        <v>110</v>
       </c>
       <c r="Q36" t="s">
-        <v>178</v>
+        <v>110</v>
       </c>
       <c r="R36" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>159</v>
+        <v>69</v>
       </c>
       <c r="B37"/>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>69</v>
+      </c>
+      <c r="D37" t="s">
+        <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="F37" t="s">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="G37" t="s">
-        <v>138</v>
-      </c>
-      <c r="J37"/>
-      <c r="K37"/>
+        <v>70</v>
+      </c>
+      <c r="H37" t="s">
+        <v>70</v>
+      </c>
+      <c r="J37" t="s">
+        <v>70</v>
+      </c>
+      <c r="K37" t="s">
+        <v>70</v>
+      </c>
+      <c r="L37" t="s">
+        <v>70</v>
+      </c>
+      <c r="M37" t="s">
+        <v>70</v>
+      </c>
       <c r="N37"/>
       <c r="O37" t="s">
         <v>129</v>
       </c>
       <c r="P37" t="s">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="Q37" t="s">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="R37" t="s">
-        <v>138</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.25">
@@ -2747,10 +2765,10 @@
         <v>108</v>
       </c>
       <c r="E38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F38" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G38" t="s">
         <v>138</v>
@@ -2762,10 +2780,10 @@
         <v>129</v>
       </c>
       <c r="P38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R38" t="s">
         <v>138</v>
@@ -2780,30 +2798,28 @@
         <v>108</v>
       </c>
       <c r="E39" t="s">
-        <v>180</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>179</v>
+        <v>101</v>
+      </c>
+      <c r="F39" t="s">
+        <v>124</v>
       </c>
       <c r="G39" t="s">
-        <v>50</v>
-      </c>
-      <c r="H39" t="s">
-        <v>38</v>
-      </c>
-      <c r="J39" s="16"/>
+        <v>138</v>
+      </c>
+      <c r="J39"/>
+      <c r="K39"/>
       <c r="N39"/>
       <c r="O39" t="s">
         <v>129</v>
       </c>
       <c r="P39" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q39" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R39" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
@@ -2812,13 +2828,13 @@
       </c>
       <c r="B40"/>
       <c r="C40" t="s">
-        <v>181</v>
+        <v>108</v>
       </c>
       <c r="E40" t="s">
-        <v>187</v>
-      </c>
-      <c r="F40" t="s">
-        <v>127</v>
+        <v>180</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>179</v>
       </c>
       <c r="G40" t="s">
         <v>50</v>
@@ -2826,23 +2842,19 @@
       <c r="H40" t="s">
         <v>38</v>
       </c>
-      <c r="J40"/>
-      <c r="K40"/>
+      <c r="J40" s="16"/>
       <c r="N40"/>
       <c r="O40" t="s">
         <v>129</v>
       </c>
       <c r="P40" t="s">
-        <v>182</v>
+        <v>114</v>
       </c>
       <c r="Q40" t="s">
-        <v>182</v>
+        <v>114</v>
       </c>
       <c r="R40" t="s">
-        <v>51</v>
-      </c>
-      <c r="T40" t="s">
-        <v>183</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
@@ -2854,10 +2866,10 @@
         <v>181</v>
       </c>
       <c r="E41" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F41" t="s">
-        <v>184</v>
+        <v>127</v>
       </c>
       <c r="G41" t="s">
         <v>50</v>
@@ -2872,10 +2884,10 @@
         <v>129</v>
       </c>
       <c r="P41" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="Q41" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="R41" t="s">
         <v>51</v>
@@ -2890,13 +2902,13 @@
       </c>
       <c r="B42"/>
       <c r="C42" t="s">
-        <v>108</v>
+        <v>181</v>
       </c>
       <c r="E42" t="s">
-        <v>102</v>
+        <v>186</v>
       </c>
       <c r="F42" t="s">
-        <v>126</v>
+        <v>184</v>
       </c>
       <c r="G42" t="s">
         <v>50</v>
@@ -2911,109 +2923,94 @@
         <v>129</v>
       </c>
       <c r="P42" t="s">
-        <v>115</v>
+        <v>185</v>
       </c>
       <c r="Q42" t="s">
-        <v>115</v>
+        <v>185</v>
       </c>
       <c r="R42" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="T42" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B43"/>
-      <c r="C43" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>134</v>
+      <c r="C43" t="s">
+        <v>108</v>
       </c>
       <c r="E43" t="s">
-        <v>167</v>
+        <v>102</v>
       </c>
       <c r="F43" t="s">
-        <v>168</v>
+        <v>126</v>
       </c>
       <c r="G43" t="s">
-        <v>51</v>
-      </c>
-      <c r="J43" s="2">
-        <v>0</v>
-      </c>
-      <c r="K43" s="17">
-        <v>1</v>
-      </c>
-      <c r="M43" t="s">
-        <v>86</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="H43" t="s">
+        <v>38</v>
+      </c>
+      <c r="J43"/>
+      <c r="K43"/>
+      <c r="N43"/>
       <c r="O43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P43" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="Q43" t="s">
-        <v>169</v>
-      </c>
-      <c r="R43" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="S43" t="s">
-        <v>78</v>
+        <v>115</v>
+      </c>
+      <c r="R43" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>160</v>
       </c>
       <c r="B44"/>
-      <c r="C44" t="s">
-        <v>69</v>
-      </c>
-      <c r="D44" t="s">
-        <v>69</v>
+      <c r="C44" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>134</v>
       </c>
       <c r="E44" t="s">
-        <v>87</v>
+        <v>167</v>
       </c>
       <c r="F44" t="s">
-        <v>88</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L44" t="s">
-        <v>70</v>
+        <v>168</v>
+      </c>
+      <c r="G44" t="s">
+        <v>51</v>
+      </c>
+      <c r="J44" s="2">
+        <v>0</v>
+      </c>
+      <c r="K44" s="17">
+        <v>1</v>
       </c>
       <c r="M44" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="O44" t="s">
         <v>130</v>
       </c>
       <c r="P44" t="s">
-        <v>87</v>
+        <v>169</v>
       </c>
       <c r="Q44" t="s">
-        <v>87</v>
-      </c>
-      <c r="R44" t="s">
-        <v>89</v>
+        <v>169</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="S44" t="s">
         <v>78</v>
@@ -3031,10 +3028,10 @@
         <v>69</v>
       </c>
       <c r="E45" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F45" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>70</v>
@@ -3061,10 +3058,10 @@
         <v>130</v>
       </c>
       <c r="P45" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="Q45" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="R45" t="s">
         <v>89</v>
@@ -3075,47 +3072,53 @@
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>160</v>
+        <v>69</v>
       </c>
       <c r="B46"/>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="D46" t="s">
-        <v>142</v>
+        <v>69</v>
       </c>
       <c r="E46" t="s">
-        <v>143</v>
+        <v>90</v>
       </c>
       <c r="F46" t="s">
-        <v>144</v>
-      </c>
-      <c r="G46" t="s">
-        <v>116</v>
-      </c>
-      <c r="J46" s="2">
-        <v>1</v>
-      </c>
-      <c r="K46" s="2">
-        <v>1</v>
+        <v>91</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="L46" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="M46" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="O46" t="s">
         <v>130</v>
       </c>
       <c r="P46" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="Q46" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="R46" t="s">
-        <v>138</v>
+        <v>89</v>
       </c>
       <c r="S46" t="s">
         <v>78</v>
@@ -3133,121 +3136,124 @@
         <v>142</v>
       </c>
       <c r="E47" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="F47" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="G47" t="s">
-        <v>50</v>
-      </c>
-      <c r="J47"/>
-      <c r="K47"/>
-      <c r="N47"/>
+        <v>116</v>
+      </c>
+      <c r="J47" s="2">
+        <v>1</v>
+      </c>
+      <c r="K47" s="2">
+        <v>1</v>
+      </c>
+      <c r="L47" t="s">
+        <v>86</v>
+      </c>
+      <c r="M47" t="s">
+        <v>78</v>
+      </c>
       <c r="O47" t="s">
         <v>130</v>
       </c>
       <c r="P47" t="s">
-        <v>161</v>
+        <v>103</v>
       </c>
       <c r="Q47" t="s">
-        <v>161</v>
+        <v>103</v>
       </c>
       <c r="R47" t="s">
-        <v>50</v>
+        <v>138</v>
+      </c>
+      <c r="S47" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>69</v>
+        <v>160</v>
       </c>
       <c r="B48"/>
       <c r="C48" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="D48" t="s">
-        <v>69</v>
-      </c>
-      <c r="E48" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L48" t="s">
-        <v>70</v>
-      </c>
-      <c r="M48" t="s">
-        <v>70</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="E48" t="s">
+        <v>162</v>
+      </c>
+      <c r="F48" t="s">
+        <v>163</v>
+      </c>
+      <c r="G48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J48"/>
+      <c r="K48"/>
+      <c r="N48"/>
       <c r="O48" t="s">
         <v>130</v>
       </c>
       <c r="P48" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="Q48" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="R48" t="s">
-        <v>138</v>
-      </c>
-      <c r="S48" t="s">
-        <v>78</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>160</v>
+        <v>69</v>
       </c>
       <c r="B49"/>
-      <c r="C49" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E49" t="s">
-        <v>135</v>
-      </c>
-      <c r="F49" t="s">
-        <v>136</v>
-      </c>
-      <c r="G49" t="s">
-        <v>138</v>
-      </c>
-      <c r="J49" s="2">
-        <v>0</v>
-      </c>
-      <c r="K49" s="17">
-        <v>1</v>
+      <c r="C49" t="s">
+        <v>69</v>
+      </c>
+      <c r="D49" t="s">
+        <v>69</v>
+      </c>
+      <c r="E49" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="L49" t="s">
+        <v>70</v>
       </c>
       <c r="M49" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="O49" t="s">
         <v>130</v>
       </c>
       <c r="P49" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="Q49" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="R49" t="s">
         <v>138</v>
@@ -3256,7 +3262,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>160</v>
       </c>
@@ -3268,10 +3274,10 @@
         <v>134</v>
       </c>
       <c r="E50" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F50" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G50" t="s">
         <v>138</v>
@@ -3289,10 +3295,10 @@
         <v>130</v>
       </c>
       <c r="P50" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="Q50" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="R50" t="s">
         <v>138</v>
@@ -3306,20 +3312,20 @@
         <v>160</v>
       </c>
       <c r="B51"/>
-      <c r="C51" t="s">
-        <v>217</v>
-      </c>
-      <c r="D51" t="s">
-        <v>211</v>
+      <c r="C51" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>134</v>
       </c>
       <c r="E51" t="s">
-        <v>170</v>
+        <v>139</v>
       </c>
       <c r="F51" t="s">
-        <v>174</v>
+        <v>140</v>
       </c>
       <c r="G51" t="s">
-        <v>175</v>
+        <v>138</v>
       </c>
       <c r="J51" s="2">
         <v>0</v>
@@ -3334,65 +3340,58 @@
         <v>130</v>
       </c>
       <c r="P51" t="s">
-        <v>210</v>
+        <v>141</v>
       </c>
       <c r="Q51" t="s">
-        <v>210</v>
-      </c>
-      <c r="R51" s="15" t="s">
-        <v>53</v>
+        <v>141</v>
+      </c>
+      <c r="R51" t="s">
+        <v>138</v>
       </c>
       <c r="S51" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>69</v>
+        <v>160</v>
       </c>
       <c r="B52"/>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>217</v>
       </c>
       <c r="D52" t="s">
-        <v>69</v>
+        <v>211</v>
       </c>
       <c r="E52" t="s">
-        <v>69</v>
+        <v>170</v>
       </c>
       <c r="F52" t="s">
-        <v>69</v>
+        <v>174</v>
       </c>
       <c r="G52" t="s">
-        <v>70</v>
-      </c>
-      <c r="H52" t="s">
-        <v>70</v>
-      </c>
-      <c r="J52" t="s">
-        <v>70</v>
-      </c>
-      <c r="K52" t="s">
-        <v>70</v>
-      </c>
-      <c r="L52" t="s">
-        <v>70</v>
+        <v>175</v>
+      </c>
+      <c r="J52" s="2">
+        <v>0</v>
+      </c>
+      <c r="K52" s="17">
+        <v>1</v>
       </c>
       <c r="M52" t="s">
-        <v>70</v>
-      </c>
-      <c r="N52"/>
+        <v>86</v>
+      </c>
       <c r="O52" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P52" t="s">
-        <v>178</v>
+        <v>210</v>
       </c>
       <c r="Q52" t="s">
-        <v>178</v>
-      </c>
-      <c r="R52" t="s">
-        <v>81</v>
+        <v>210</v>
+      </c>
+      <c r="R52" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="S52" t="s">
         <v>78</v>
@@ -3438,52 +3437,65 @@
         <v>131</v>
       </c>
       <c r="P53" t="s">
-        <v>219</v>
+        <v>178</v>
       </c>
       <c r="Q53" t="s">
-        <v>219</v>
+        <v>178</v>
       </c>
       <c r="R53" t="s">
-        <v>220</v>
+        <v>81</v>
       </c>
       <c r="S53" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>159</v>
+      <c r="A54" t="s">
+        <v>69</v>
       </c>
       <c r="B54"/>
       <c r="C54" t="s">
-        <v>215</v>
+        <v>69</v>
       </c>
       <c r="D54" t="s">
-        <v>218</v>
+        <v>69</v>
       </c>
       <c r="E54" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="F54" t="s">
-        <v>118</v>
+        <v>69</v>
       </c>
       <c r="G54" t="s">
-        <v>138</v>
-      </c>
-      <c r="J54"/>
-      <c r="K54"/>
+        <v>70</v>
+      </c>
+      <c r="H54" t="s">
+        <v>70</v>
+      </c>
+      <c r="J54" t="s">
+        <v>70</v>
+      </c>
+      <c r="K54" t="s">
+        <v>70</v>
+      </c>
+      <c r="L54" t="s">
+        <v>70</v>
+      </c>
+      <c r="M54" t="s">
+        <v>70</v>
+      </c>
       <c r="N54"/>
       <c r="O54" t="s">
         <v>131</v>
       </c>
       <c r="P54" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="Q54" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="R54" t="s">
-        <v>138</v>
+        <v>220</v>
       </c>
       <c r="S54" t="s">
         <v>78</v>
@@ -3501,10 +3513,10 @@
         <v>218</v>
       </c>
       <c r="E55" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F55" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G55" t="s">
         <v>138</v>
@@ -3516,10 +3528,10 @@
         <v>131</v>
       </c>
       <c r="P55" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="Q55" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R55" t="s">
         <v>138</v>
@@ -3534,19 +3546,19 @@
       </c>
       <c r="B56"/>
       <c r="C56" t="s">
-        <v>145</v>
+        <v>215</v>
       </c>
       <c r="D56" t="s">
-        <v>146</v>
+        <v>218</v>
       </c>
       <c r="E56" t="s">
-        <v>221</v>
+        <v>96</v>
       </c>
       <c r="F56" t="s">
-        <v>222</v>
+        <v>119</v>
       </c>
       <c r="G56" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
       <c r="J56"/>
       <c r="K56"/>
@@ -3555,13 +3567,13 @@
         <v>131</v>
       </c>
       <c r="P56" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="Q56" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="R56" t="s">
-        <v>50</v>
+        <v>138</v>
       </c>
       <c r="S56" t="s">
         <v>78</v>
@@ -3573,19 +3585,19 @@
       </c>
       <c r="B57"/>
       <c r="C57" t="s">
-        <v>145</v>
+        <v>228</v>
       </c>
       <c r="D57" t="s">
-        <v>146</v>
+        <v>229</v>
       </c>
       <c r="E57" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="F57" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="G57" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="J57"/>
       <c r="K57"/>
@@ -3594,13 +3606,13 @@
         <v>131</v>
       </c>
       <c r="P57" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="Q57" t="s">
-        <v>148</v>
-      </c>
-      <c r="R57" t="s">
-        <v>81</v>
+        <v>169</v>
+      </c>
+      <c r="R57" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="S57" t="s">
         <v>78</v>
@@ -3618,13 +3630,13 @@
         <v>146</v>
       </c>
       <c r="E58" t="s">
-        <v>149</v>
+        <v>221</v>
       </c>
       <c r="F58" t="s">
-        <v>150</v>
+        <v>222</v>
       </c>
       <c r="G58" t="s">
-        <v>151</v>
+        <v>50</v>
       </c>
       <c r="J58"/>
       <c r="K58"/>
@@ -3633,13 +3645,13 @@
         <v>131</v>
       </c>
       <c r="P58" t="s">
-        <v>152</v>
+        <v>223</v>
       </c>
       <c r="Q58" t="s">
-        <v>152</v>
+        <v>223</v>
       </c>
       <c r="R58" t="s">
-        <v>151</v>
+        <v>50</v>
       </c>
       <c r="S58" t="s">
         <v>78</v>
@@ -3657,13 +3669,13 @@
         <v>146</v>
       </c>
       <c r="E59" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F59" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G59" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="J59"/>
       <c r="K59"/>
@@ -3672,13 +3684,13 @@
         <v>131</v>
       </c>
       <c r="P59" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="Q59" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="R59" t="s">
-        <v>50</v>
+        <v>226</v>
       </c>
       <c r="S59" t="s">
         <v>78</v>
@@ -3696,10 +3708,10 @@
         <v>146</v>
       </c>
       <c r="E60" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F60" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="G60" t="s">
         <v>151</v>
@@ -3711,10 +3723,10 @@
         <v>131</v>
       </c>
       <c r="P60" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="Q60" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="R60" t="s">
         <v>151</v>
@@ -3735,10 +3747,10 @@
         <v>146</v>
       </c>
       <c r="E61" t="s">
-        <v>207</v>
+        <v>153</v>
       </c>
       <c r="F61" t="s">
-        <v>208</v>
+        <v>154</v>
       </c>
       <c r="G61" t="s">
         <v>50</v>
@@ -3750,238 +3762,302 @@
         <v>131</v>
       </c>
       <c r="P61" t="s">
-        <v>209</v>
+        <v>155</v>
       </c>
       <c r="Q61" t="s">
-        <v>209</v>
+        <v>155</v>
       </c>
       <c r="R61" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="S61" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>160</v>
+      <c r="A62" s="1" t="s">
+        <v>159</v>
       </c>
       <c r="B62"/>
       <c r="C62" t="s">
-        <v>55</v>
+        <v>145</v>
       </c>
       <c r="D62" t="s">
-        <v>35</v>
+        <v>146</v>
       </c>
       <c r="E62" t="s">
-        <v>5</v>
+        <v>156</v>
       </c>
       <c r="F62" t="s">
-        <v>33</v>
+        <v>157</v>
       </c>
       <c r="G62" t="s">
-        <v>50</v>
-      </c>
-      <c r="H62" t="s">
-        <v>38</v>
-      </c>
-      <c r="J62">
-        <v>0</v>
-      </c>
-      <c r="K62" t="s">
-        <v>7</v>
-      </c>
-      <c r="N62" t="s">
-        <v>43</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="J62"/>
+      <c r="K62"/>
+      <c r="N62"/>
       <c r="O62" t="s">
-        <v>41</v>
+        <v>131</v>
       </c>
       <c r="P62" t="s">
-        <v>52</v>
+        <v>158</v>
       </c>
       <c r="Q62" t="s">
-        <v>52</v>
+        <v>158</v>
       </c>
       <c r="R62" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="S62" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="63" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B63"/>
+      <c r="C63" t="s">
+        <v>145</v>
+      </c>
+      <c r="D63" t="s">
+        <v>146</v>
+      </c>
+      <c r="E63" t="s">
+        <v>207</v>
+      </c>
+      <c r="F63" t="s">
+        <v>208</v>
+      </c>
+      <c r="G63" t="s">
+        <v>50</v>
+      </c>
+      <c r="J63"/>
+      <c r="K63"/>
+      <c r="N63"/>
+      <c r="O63" t="s">
+        <v>131</v>
+      </c>
+      <c r="P63" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>209</v>
+      </c>
+      <c r="R63" t="s">
+        <v>227</v>
+      </c>
+      <c r="S63" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>160</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="B64"/>
+      <c r="C64" t="s">
         <v>55</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="D64" t="s">
         <v>35</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E64" t="s">
+        <v>5</v>
+      </c>
+      <c r="F64" t="s">
+        <v>33</v>
+      </c>
+      <c r="G64" t="s">
+        <v>50</v>
+      </c>
+      <c r="H64" t="s">
+        <v>38</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+      <c r="K64" t="s">
+        <v>7</v>
+      </c>
+      <c r="N64" t="s">
+        <v>43</v>
+      </c>
+      <c r="O64" t="s">
+        <v>41</v>
+      </c>
+      <c r="P64" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>52</v>
+      </c>
+      <c r="R64" t="s">
+        <v>50</v>
+      </c>
+      <c r="S64" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>160</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="F65" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G63" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="H65" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J65" s="1">
         <v>0</v>
       </c>
-      <c r="K63" s="1" t="s">
+      <c r="K65" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N63" s="1" t="s">
+      <c r="N65" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="O63" s="1" t="s">
+      <c r="O65" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="P63" s="1" t="s">
+      <c r="P65" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="Q63" s="1" t="s">
+      <c r="Q65" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="R63" s="1" t="s">
+      <c r="R65" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="S63" s="1" t="s">
+      <c r="S65" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="64" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G64" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="K64" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="L64" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="M64" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="O64" s="1" t="s">
+    <row r="66" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="K66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="O66" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="P64" s="1" t="s">
+      <c r="P66" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="Q64" s="1" t="s">
+      <c r="Q66" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="R64" s="1" t="s">
+      <c r="R66" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="S64" s="1" t="s">
+      <c r="S66" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="65" spans="1:20" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F65" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="G65" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="H65" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="I65" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="J65" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="K65" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="L65" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="M65" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="N65" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="O65" s="6" t="s">
+    <row r="67" spans="1:20" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G67" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H67" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="I67" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="J67" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="K67" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="L67" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="N67" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="O67" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="P65" s="6" t="s">
+      <c r="P67" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="Q65" s="6" t="s">
+      <c r="Q67" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="R65" s="6" t="s">
+      <c r="R67" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="S65" s="6" t="s">
+      <c r="S67" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="T65" s="6" t="s">
+      <c r="T67" s="6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A66"/>
-      <c r="B66"/>
-      <c r="J66"/>
-      <c r="K66"/>
-      <c r="N66"/>
-    </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A67"/>
-      <c r="B67"/>
-      <c r="J67"/>
-      <c r="K67"/>
-      <c r="N67"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68"/>
@@ -4074,198 +4150,1352 @@
       <c r="K80"/>
       <c r="N80"/>
     </row>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="84" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="85" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="86" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="87" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="88" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="89" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="90" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="91" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="92" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="93" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="94" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="95" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="96" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="97" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="98" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="99" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="100" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="101" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="102" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="103" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="104" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="105" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="106" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="107" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="108" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="109" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="110" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="111" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="112" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="113" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="114" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="115" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="116" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="117" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="118" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="119" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="120" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="121" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="122" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="123" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="124" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="125" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="126" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="127" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="128" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="129" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="130" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="131" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="132" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="133" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="134" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="135" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="136" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="137" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="138" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="139" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="140" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="141" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="142" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="143" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="144" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="145" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="146" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="147" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="148" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="149" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="150" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="151" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="152" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="153" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="154" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="155" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="156" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="157" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="158" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="159" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="160" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="161" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="162" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="163" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="164" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="165" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="166" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="167" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="168" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="169" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="170" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="171" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="172" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="173" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="174" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="175" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="176" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="177" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="178" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="179" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="180" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="181" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="182" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="183" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="184" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="185" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="186" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="187" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="188" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="189" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="190" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="191" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="192" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="193" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="194" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="195" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="196" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="197" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="198" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="199" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="200" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="201" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="202" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="203" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="204" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="205" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="206" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="207" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="208" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="209" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="210" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="211" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="212" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="213" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="214" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="215" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="216" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="217" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="218" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="219" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="220" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="221" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="222" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="223" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="224" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="225" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="226" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="227" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="228" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="229" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="230" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="231" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="232" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="233" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="234" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="235" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="236" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="237" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="238" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="239" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="240" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="241" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="242" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="243" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="244" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="245" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="246" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="247" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="248" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="249" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="250" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="251" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="252" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="253" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="254" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="255" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="256" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="257" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="258" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="259" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="260" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="261" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="262" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="263" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="264" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="265" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="266" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="267" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="268" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="269" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="270" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A81"/>
+      <c r="B81"/>
+      <c r="J81"/>
+      <c r="K81"/>
+      <c r="N81"/>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A82"/>
+      <c r="B82"/>
+      <c r="J82"/>
+      <c r="K82"/>
+      <c r="N82"/>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A83"/>
+      <c r="B83"/>
+      <c r="J83"/>
+      <c r="K83"/>
+      <c r="N83"/>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A84"/>
+      <c r="B84"/>
+      <c r="J84"/>
+      <c r="K84"/>
+      <c r="N84"/>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A85"/>
+      <c r="B85"/>
+      <c r="J85"/>
+      <c r="K85"/>
+      <c r="N85"/>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86"/>
+      <c r="B86"/>
+      <c r="J86"/>
+      <c r="K86"/>
+      <c r="N86"/>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A87"/>
+      <c r="B87"/>
+      <c r="J87"/>
+      <c r="K87"/>
+      <c r="N87"/>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A88"/>
+      <c r="B88"/>
+      <c r="J88"/>
+      <c r="K88"/>
+      <c r="N88"/>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89"/>
+      <c r="B89"/>
+      <c r="J89"/>
+      <c r="K89"/>
+      <c r="N89"/>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90"/>
+      <c r="B90"/>
+      <c r="J90"/>
+      <c r="K90"/>
+      <c r="N90"/>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91"/>
+      <c r="B91"/>
+      <c r="J91"/>
+      <c r="K91"/>
+      <c r="N91"/>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92"/>
+      <c r="B92"/>
+      <c r="J92"/>
+      <c r="K92"/>
+      <c r="N92"/>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93"/>
+      <c r="B93"/>
+      <c r="J93"/>
+      <c r="K93"/>
+      <c r="N93"/>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94"/>
+      <c r="B94"/>
+      <c r="J94"/>
+      <c r="K94"/>
+      <c r="N94"/>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95"/>
+      <c r="B95"/>
+      <c r="J95"/>
+      <c r="K95"/>
+      <c r="N95"/>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96"/>
+      <c r="B96"/>
+      <c r="J96"/>
+      <c r="K96"/>
+      <c r="N96"/>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97"/>
+      <c r="B97"/>
+      <c r="J97"/>
+      <c r="K97"/>
+      <c r="N97"/>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98"/>
+      <c r="B98"/>
+      <c r="J98"/>
+      <c r="K98"/>
+      <c r="N98"/>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99"/>
+      <c r="B99"/>
+      <c r="J99"/>
+      <c r="K99"/>
+      <c r="N99"/>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100"/>
+      <c r="B100"/>
+      <c r="J100"/>
+      <c r="K100"/>
+      <c r="N100"/>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A101"/>
+      <c r="B101"/>
+      <c r="J101"/>
+      <c r="K101"/>
+      <c r="N101"/>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A102"/>
+      <c r="B102"/>
+      <c r="J102"/>
+      <c r="K102"/>
+      <c r="N102"/>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A103"/>
+      <c r="B103"/>
+      <c r="J103"/>
+      <c r="K103"/>
+      <c r="N103"/>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A104"/>
+      <c r="B104"/>
+      <c r="J104"/>
+      <c r="K104"/>
+      <c r="N104"/>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A105"/>
+      <c r="B105"/>
+      <c r="J105"/>
+      <c r="K105"/>
+      <c r="N105"/>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106"/>
+      <c r="B106"/>
+      <c r="J106"/>
+      <c r="K106"/>
+      <c r="N106"/>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A107"/>
+      <c r="B107"/>
+      <c r="J107"/>
+      <c r="K107"/>
+      <c r="N107"/>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108"/>
+      <c r="B108"/>
+      <c r="J108"/>
+      <c r="K108"/>
+      <c r="N108"/>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A109"/>
+      <c r="B109"/>
+      <c r="J109"/>
+      <c r="K109"/>
+      <c r="N109"/>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A110"/>
+      <c r="B110"/>
+      <c r="J110"/>
+      <c r="K110"/>
+      <c r="N110"/>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A111"/>
+      <c r="B111"/>
+      <c r="J111"/>
+      <c r="K111"/>
+      <c r="N111"/>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A112"/>
+      <c r="B112"/>
+      <c r="J112"/>
+      <c r="K112"/>
+      <c r="N112"/>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A113"/>
+      <c r="B113"/>
+      <c r="J113"/>
+      <c r="K113"/>
+      <c r="N113"/>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A114"/>
+      <c r="B114"/>
+      <c r="J114"/>
+      <c r="K114"/>
+      <c r="N114"/>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A115"/>
+      <c r="B115"/>
+      <c r="J115"/>
+      <c r="K115"/>
+      <c r="N115"/>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A116"/>
+      <c r="B116"/>
+      <c r="J116"/>
+      <c r="K116"/>
+      <c r="N116"/>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A117"/>
+      <c r="B117"/>
+      <c r="J117"/>
+      <c r="K117"/>
+      <c r="N117"/>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A118"/>
+      <c r="B118"/>
+      <c r="J118"/>
+      <c r="K118"/>
+      <c r="N118"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A119"/>
+      <c r="B119"/>
+      <c r="J119"/>
+      <c r="K119"/>
+      <c r="N119"/>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A120"/>
+      <c r="B120"/>
+      <c r="J120"/>
+      <c r="K120"/>
+      <c r="N120"/>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A121"/>
+      <c r="B121"/>
+      <c r="J121"/>
+      <c r="K121"/>
+      <c r="N121"/>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A122"/>
+      <c r="B122"/>
+      <c r="J122"/>
+      <c r="K122"/>
+      <c r="N122"/>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A123"/>
+      <c r="B123"/>
+      <c r="J123"/>
+      <c r="K123"/>
+      <c r="N123"/>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A124"/>
+      <c r="B124"/>
+      <c r="J124"/>
+      <c r="K124"/>
+      <c r="N124"/>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A125"/>
+      <c r="B125"/>
+      <c r="J125"/>
+      <c r="K125"/>
+      <c r="N125"/>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A126"/>
+      <c r="B126"/>
+      <c r="J126"/>
+      <c r="K126"/>
+      <c r="N126"/>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127"/>
+      <c r="B127"/>
+      <c r="J127"/>
+      <c r="K127"/>
+      <c r="N127"/>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A128"/>
+      <c r="B128"/>
+      <c r="J128"/>
+      <c r="K128"/>
+      <c r="N128"/>
+    </row>
+    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A129"/>
+      <c r="B129"/>
+      <c r="J129"/>
+      <c r="K129"/>
+      <c r="N129"/>
+    </row>
+    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A130"/>
+      <c r="B130"/>
+      <c r="J130"/>
+      <c r="K130"/>
+      <c r="N130"/>
+    </row>
+    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A131"/>
+      <c r="B131"/>
+      <c r="J131"/>
+      <c r="K131"/>
+      <c r="N131"/>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A132"/>
+      <c r="B132"/>
+      <c r="J132"/>
+      <c r="K132"/>
+      <c r="N132"/>
+    </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A133"/>
+      <c r="B133"/>
+      <c r="J133"/>
+      <c r="K133"/>
+      <c r="N133"/>
+    </row>
+    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A134"/>
+      <c r="B134"/>
+      <c r="J134"/>
+      <c r="K134"/>
+      <c r="N134"/>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A135"/>
+      <c r="B135"/>
+      <c r="J135"/>
+      <c r="K135"/>
+      <c r="N135"/>
+    </row>
+    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A136"/>
+      <c r="B136"/>
+      <c r="J136"/>
+      <c r="K136"/>
+      <c r="N136"/>
+    </row>
+    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A137"/>
+      <c r="B137"/>
+      <c r="J137"/>
+      <c r="K137"/>
+      <c r="N137"/>
+    </row>
+    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A138"/>
+      <c r="B138"/>
+      <c r="J138"/>
+      <c r="K138"/>
+      <c r="N138"/>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A139"/>
+      <c r="B139"/>
+      <c r="J139"/>
+      <c r="K139"/>
+      <c r="N139"/>
+    </row>
+    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A140"/>
+      <c r="B140"/>
+      <c r="J140"/>
+      <c r="K140"/>
+      <c r="N140"/>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A141"/>
+      <c r="B141"/>
+      <c r="J141"/>
+      <c r="K141"/>
+      <c r="N141"/>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A142"/>
+      <c r="B142"/>
+      <c r="J142"/>
+      <c r="K142"/>
+      <c r="N142"/>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A143"/>
+      <c r="B143"/>
+      <c r="J143"/>
+      <c r="K143"/>
+      <c r="N143"/>
+    </row>
+    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A144"/>
+      <c r="B144"/>
+      <c r="J144"/>
+      <c r="K144"/>
+      <c r="N144"/>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A145"/>
+      <c r="B145"/>
+      <c r="J145"/>
+      <c r="K145"/>
+      <c r="N145"/>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A146"/>
+      <c r="B146"/>
+      <c r="J146"/>
+      <c r="K146"/>
+      <c r="N146"/>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A147"/>
+      <c r="B147"/>
+      <c r="J147"/>
+      <c r="K147"/>
+      <c r="N147"/>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A148"/>
+      <c r="B148"/>
+      <c r="J148"/>
+      <c r="K148"/>
+      <c r="N148"/>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A149"/>
+      <c r="B149"/>
+      <c r="J149"/>
+      <c r="K149"/>
+      <c r="N149"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A150"/>
+      <c r="B150"/>
+      <c r="J150"/>
+      <c r="K150"/>
+      <c r="N150"/>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A151"/>
+      <c r="B151"/>
+      <c r="J151"/>
+      <c r="K151"/>
+      <c r="N151"/>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A152"/>
+      <c r="B152"/>
+      <c r="J152"/>
+      <c r="K152"/>
+      <c r="N152"/>
+    </row>
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A153"/>
+      <c r="B153"/>
+      <c r="J153"/>
+      <c r="K153"/>
+      <c r="N153"/>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A154"/>
+      <c r="B154"/>
+      <c r="J154"/>
+      <c r="K154"/>
+      <c r="N154"/>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A155"/>
+      <c r="B155"/>
+      <c r="J155"/>
+      <c r="K155"/>
+      <c r="N155"/>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A156"/>
+      <c r="B156"/>
+      <c r="J156"/>
+      <c r="K156"/>
+      <c r="N156"/>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A157"/>
+      <c r="B157"/>
+      <c r="J157"/>
+      <c r="K157"/>
+      <c r="N157"/>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A158"/>
+      <c r="B158"/>
+      <c r="J158"/>
+      <c r="K158"/>
+      <c r="N158"/>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A159"/>
+      <c r="B159"/>
+      <c r="J159"/>
+      <c r="K159"/>
+      <c r="N159"/>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A160"/>
+      <c r="B160"/>
+      <c r="J160"/>
+      <c r="K160"/>
+      <c r="N160"/>
+    </row>
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A161"/>
+      <c r="B161"/>
+      <c r="J161"/>
+      <c r="K161"/>
+      <c r="N161"/>
+    </row>
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A162"/>
+      <c r="B162"/>
+      <c r="J162"/>
+      <c r="K162"/>
+      <c r="N162"/>
+    </row>
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A163"/>
+      <c r="B163"/>
+      <c r="J163"/>
+      <c r="K163"/>
+      <c r="N163"/>
+    </row>
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A164"/>
+      <c r="B164"/>
+      <c r="J164"/>
+      <c r="K164"/>
+      <c r="N164"/>
+    </row>
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A165"/>
+      <c r="B165"/>
+      <c r="J165"/>
+      <c r="K165"/>
+      <c r="N165"/>
+    </row>
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A166"/>
+      <c r="B166"/>
+      <c r="J166"/>
+      <c r="K166"/>
+      <c r="N166"/>
+    </row>
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A167"/>
+      <c r="B167"/>
+      <c r="J167"/>
+      <c r="K167"/>
+      <c r="N167"/>
+    </row>
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A168"/>
+      <c r="B168"/>
+      <c r="J168"/>
+      <c r="K168"/>
+      <c r="N168"/>
+    </row>
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A169"/>
+      <c r="B169"/>
+      <c r="J169"/>
+      <c r="K169"/>
+      <c r="N169"/>
+    </row>
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A170"/>
+      <c r="B170"/>
+      <c r="J170"/>
+      <c r="K170"/>
+      <c r="N170"/>
+    </row>
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A171"/>
+      <c r="B171"/>
+      <c r="J171"/>
+      <c r="K171"/>
+      <c r="N171"/>
+    </row>
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A172"/>
+      <c r="B172"/>
+      <c r="J172"/>
+      <c r="K172"/>
+      <c r="N172"/>
+    </row>
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A173"/>
+      <c r="B173"/>
+      <c r="J173"/>
+      <c r="K173"/>
+      <c r="N173"/>
+    </row>
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A174"/>
+      <c r="B174"/>
+      <c r="J174"/>
+      <c r="K174"/>
+      <c r="N174"/>
+    </row>
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A175"/>
+      <c r="B175"/>
+      <c r="J175"/>
+      <c r="K175"/>
+      <c r="N175"/>
+    </row>
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A176"/>
+      <c r="B176"/>
+      <c r="J176"/>
+      <c r="K176"/>
+      <c r="N176"/>
+    </row>
+    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A177"/>
+      <c r="B177"/>
+      <c r="J177"/>
+      <c r="K177"/>
+      <c r="N177"/>
+    </row>
+    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A178"/>
+      <c r="B178"/>
+      <c r="J178"/>
+      <c r="K178"/>
+      <c r="N178"/>
+    </row>
+    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A179"/>
+      <c r="B179"/>
+      <c r="J179"/>
+      <c r="K179"/>
+      <c r="N179"/>
+    </row>
+    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A180"/>
+      <c r="B180"/>
+      <c r="J180"/>
+      <c r="K180"/>
+      <c r="N180"/>
+    </row>
+    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A181"/>
+      <c r="B181"/>
+      <c r="J181"/>
+      <c r="K181"/>
+      <c r="N181"/>
+    </row>
+    <row r="182" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A182"/>
+      <c r="B182"/>
+      <c r="J182"/>
+      <c r="K182"/>
+      <c r="N182"/>
+    </row>
+    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A183"/>
+      <c r="B183"/>
+      <c r="J183"/>
+      <c r="K183"/>
+      <c r="N183"/>
+    </row>
+    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A184"/>
+      <c r="B184"/>
+      <c r="J184"/>
+      <c r="K184"/>
+      <c r="N184"/>
+    </row>
+    <row r="185" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A185"/>
+      <c r="B185"/>
+      <c r="J185"/>
+      <c r="K185"/>
+      <c r="N185"/>
+    </row>
+    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A186"/>
+      <c r="B186"/>
+      <c r="J186"/>
+      <c r="K186"/>
+      <c r="N186"/>
+    </row>
+    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A187"/>
+      <c r="B187"/>
+      <c r="J187"/>
+      <c r="K187"/>
+      <c r="N187"/>
+    </row>
+    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A188"/>
+      <c r="B188"/>
+      <c r="J188"/>
+      <c r="K188"/>
+      <c r="N188"/>
+    </row>
+    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A189"/>
+      <c r="B189"/>
+      <c r="J189"/>
+      <c r="K189"/>
+      <c r="N189"/>
+    </row>
+    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A190"/>
+      <c r="B190"/>
+      <c r="J190"/>
+      <c r="K190"/>
+      <c r="N190"/>
+    </row>
+    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A191"/>
+      <c r="B191"/>
+      <c r="J191"/>
+      <c r="K191"/>
+      <c r="N191"/>
+    </row>
+    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A192"/>
+      <c r="B192"/>
+      <c r="J192"/>
+      <c r="K192"/>
+      <c r="N192"/>
+    </row>
+    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A193"/>
+      <c r="B193"/>
+      <c r="J193"/>
+      <c r="K193"/>
+      <c r="N193"/>
+    </row>
+    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A194"/>
+      <c r="B194"/>
+      <c r="J194"/>
+      <c r="K194"/>
+      <c r="N194"/>
+    </row>
+    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A195"/>
+      <c r="B195"/>
+      <c r="J195"/>
+      <c r="K195"/>
+      <c r="N195"/>
+    </row>
+    <row r="196" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A196"/>
+      <c r="B196"/>
+      <c r="J196"/>
+      <c r="K196"/>
+      <c r="N196"/>
+    </row>
+    <row r="197" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A197"/>
+      <c r="B197"/>
+      <c r="J197"/>
+      <c r="K197"/>
+      <c r="N197"/>
+    </row>
+    <row r="198" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A198"/>
+      <c r="B198"/>
+      <c r="J198"/>
+      <c r="K198"/>
+      <c r="N198"/>
+    </row>
+    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A199"/>
+      <c r="B199"/>
+      <c r="J199"/>
+      <c r="K199"/>
+      <c r="N199"/>
+    </row>
+    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A200"/>
+      <c r="B200"/>
+      <c r="J200"/>
+      <c r="K200"/>
+      <c r="N200"/>
+    </row>
+    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A201"/>
+      <c r="B201"/>
+      <c r="J201"/>
+      <c r="K201"/>
+      <c r="N201"/>
+    </row>
+    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A202"/>
+      <c r="B202"/>
+      <c r="J202"/>
+      <c r="K202"/>
+      <c r="N202"/>
+    </row>
+    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A203"/>
+      <c r="B203"/>
+      <c r="J203"/>
+      <c r="K203"/>
+      <c r="N203"/>
+    </row>
+    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A204"/>
+      <c r="B204"/>
+      <c r="J204"/>
+      <c r="K204"/>
+      <c r="N204"/>
+    </row>
+    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A205"/>
+      <c r="B205"/>
+      <c r="J205"/>
+      <c r="K205"/>
+      <c r="N205"/>
+    </row>
+    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A206"/>
+      <c r="B206"/>
+      <c r="J206"/>
+      <c r="K206"/>
+      <c r="N206"/>
+    </row>
+    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A207"/>
+      <c r="B207"/>
+      <c r="J207"/>
+      <c r="K207"/>
+      <c r="N207"/>
+    </row>
+    <row r="208" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A208"/>
+      <c r="B208"/>
+      <c r="J208"/>
+      <c r="K208"/>
+      <c r="N208"/>
+    </row>
+    <row r="209" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A209"/>
+      <c r="B209"/>
+      <c r="J209"/>
+      <c r="K209"/>
+      <c r="N209"/>
+    </row>
+    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A210"/>
+      <c r="B210"/>
+      <c r="J210"/>
+      <c r="K210"/>
+      <c r="N210"/>
+    </row>
+    <row r="211" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A211"/>
+      <c r="B211"/>
+      <c r="J211"/>
+      <c r="K211"/>
+      <c r="N211"/>
+    </row>
+    <row r="212" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A212"/>
+      <c r="B212"/>
+      <c r="J212"/>
+      <c r="K212"/>
+      <c r="N212"/>
+    </row>
+    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A213"/>
+      <c r="B213"/>
+      <c r="J213"/>
+      <c r="K213"/>
+      <c r="N213"/>
+    </row>
+    <row r="214" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A214"/>
+      <c r="B214"/>
+      <c r="J214"/>
+      <c r="K214"/>
+      <c r="N214"/>
+    </row>
+    <row r="215" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A215"/>
+      <c r="B215"/>
+      <c r="J215"/>
+      <c r="K215"/>
+      <c r="N215"/>
+    </row>
+    <row r="216" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A216"/>
+      <c r="B216"/>
+      <c r="J216"/>
+      <c r="K216"/>
+      <c r="N216"/>
+    </row>
+    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A217"/>
+      <c r="B217"/>
+      <c r="J217"/>
+      <c r="K217"/>
+      <c r="N217"/>
+    </row>
+    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A218"/>
+      <c r="B218"/>
+      <c r="J218"/>
+      <c r="K218"/>
+      <c r="N218"/>
+    </row>
+    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A219"/>
+      <c r="B219"/>
+      <c r="J219"/>
+      <c r="K219"/>
+      <c r="N219"/>
+    </row>
+    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A220"/>
+      <c r="B220"/>
+      <c r="J220"/>
+      <c r="K220"/>
+      <c r="N220"/>
+    </row>
+    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A221"/>
+      <c r="B221"/>
+      <c r="J221"/>
+      <c r="K221"/>
+      <c r="N221"/>
+    </row>
+    <row r="222" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A222"/>
+      <c r="B222"/>
+      <c r="J222"/>
+      <c r="K222"/>
+      <c r="N222"/>
+    </row>
+    <row r="223" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A223"/>
+      <c r="B223"/>
+      <c r="J223"/>
+      <c r="K223"/>
+      <c r="N223"/>
+    </row>
+    <row r="224" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A224"/>
+      <c r="B224"/>
+      <c r="J224"/>
+      <c r="K224"/>
+      <c r="N224"/>
+    </row>
+    <row r="225" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A225"/>
+      <c r="B225"/>
+      <c r="J225"/>
+      <c r="K225"/>
+      <c r="N225"/>
+    </row>
+    <row r="226" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A226"/>
+      <c r="B226"/>
+      <c r="J226"/>
+      <c r="K226"/>
+      <c r="N226"/>
+    </row>
+    <row r="227" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A227"/>
+      <c r="B227"/>
+      <c r="J227"/>
+      <c r="K227"/>
+      <c r="N227"/>
+    </row>
+    <row r="228" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A228"/>
+      <c r="B228"/>
+      <c r="J228"/>
+      <c r="K228"/>
+      <c r="N228"/>
+    </row>
+    <row r="229" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A229"/>
+      <c r="B229"/>
+      <c r="J229"/>
+      <c r="K229"/>
+      <c r="N229"/>
+    </row>
+    <row r="230" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A230"/>
+      <c r="B230"/>
+      <c r="J230"/>
+      <c r="K230"/>
+      <c r="N230"/>
+    </row>
+    <row r="231" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A231"/>
+      <c r="B231"/>
+      <c r="J231"/>
+      <c r="K231"/>
+      <c r="N231"/>
+    </row>
+    <row r="232" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A232"/>
+      <c r="B232"/>
+      <c r="J232"/>
+      <c r="K232"/>
+      <c r="N232"/>
+    </row>
+    <row r="233" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A233"/>
+      <c r="B233"/>
+      <c r="J233"/>
+      <c r="K233"/>
+      <c r="N233"/>
+    </row>
+    <row r="234" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A234"/>
+      <c r="B234"/>
+      <c r="J234"/>
+      <c r="K234"/>
+      <c r="N234"/>
+    </row>
+    <row r="235" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A235"/>
+      <c r="B235"/>
+      <c r="J235"/>
+      <c r="K235"/>
+      <c r="N235"/>
+    </row>
+    <row r="236" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A236"/>
+      <c r="B236"/>
+      <c r="J236"/>
+      <c r="K236"/>
+      <c r="N236"/>
+    </row>
+    <row r="237" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A237"/>
+      <c r="B237"/>
+      <c r="J237"/>
+      <c r="K237"/>
+      <c r="N237"/>
+    </row>
+    <row r="238" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A238"/>
+      <c r="B238"/>
+      <c r="J238"/>
+      <c r="K238"/>
+      <c r="N238"/>
+    </row>
+    <row r="239" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A239"/>
+      <c r="B239"/>
+      <c r="J239"/>
+      <c r="K239"/>
+      <c r="N239"/>
+    </row>
+    <row r="240" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A240"/>
+      <c r="B240"/>
+      <c r="J240"/>
+      <c r="K240"/>
+      <c r="N240"/>
+    </row>
+    <row r="241" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A241"/>
+      <c r="B241"/>
+      <c r="J241"/>
+      <c r="K241"/>
+      <c r="N241"/>
+    </row>
+    <row r="242" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A242"/>
+      <c r="B242"/>
+      <c r="J242"/>
+      <c r="K242"/>
+      <c r="N242"/>
+    </row>
+    <row r="243" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A243"/>
+      <c r="B243"/>
+      <c r="J243"/>
+      <c r="K243"/>
+      <c r="N243"/>
+    </row>
+    <row r="244" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A244"/>
+      <c r="B244"/>
+      <c r="J244"/>
+      <c r="K244"/>
+      <c r="N244"/>
+    </row>
+    <row r="245" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A245"/>
+      <c r="B245"/>
+      <c r="J245"/>
+      <c r="K245"/>
+      <c r="N245"/>
+    </row>
+    <row r="246" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A246"/>
+      <c r="B246"/>
+      <c r="J246"/>
+      <c r="K246"/>
+      <c r="N246"/>
+    </row>
+    <row r="247" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A247"/>
+      <c r="B247"/>
+      <c r="J247"/>
+      <c r="K247"/>
+      <c r="N247"/>
+    </row>
+    <row r="248" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A248"/>
+      <c r="B248"/>
+      <c r="J248"/>
+      <c r="K248"/>
+      <c r="N248"/>
+    </row>
+    <row r="249" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A249"/>
+      <c r="B249"/>
+      <c r="J249"/>
+      <c r="K249"/>
+      <c r="N249"/>
+    </row>
+    <row r="250" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A250"/>
+      <c r="B250"/>
+      <c r="J250"/>
+      <c r="K250"/>
+      <c r="N250"/>
+    </row>
+    <row r="251" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A251"/>
+      <c r="B251"/>
+      <c r="J251"/>
+      <c r="K251"/>
+      <c r="N251"/>
+    </row>
+    <row r="252" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A252"/>
+      <c r="B252"/>
+      <c r="J252"/>
+      <c r="K252"/>
+      <c r="N252"/>
+    </row>
+    <row r="253" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A253"/>
+      <c r="B253"/>
+      <c r="J253"/>
+      <c r="K253"/>
+      <c r="N253"/>
+    </row>
+    <row r="254" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A254"/>
+      <c r="B254"/>
+      <c r="J254"/>
+      <c r="K254"/>
+      <c r="N254"/>
+    </row>
+    <row r="255" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A255"/>
+      <c r="B255"/>
+      <c r="J255"/>
+      <c r="K255"/>
+      <c r="N255"/>
+    </row>
+    <row r="256" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A256"/>
+      <c r="B256"/>
+      <c r="J256"/>
+      <c r="K256"/>
+      <c r="N256"/>
+    </row>
+    <row r="257" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A257"/>
+      <c r="B257"/>
+      <c r="J257"/>
+      <c r="K257"/>
+      <c r="N257"/>
+    </row>
+    <row r="258" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A258"/>
+      <c r="B258"/>
+      <c r="J258"/>
+      <c r="K258"/>
+      <c r="N258"/>
+    </row>
+    <row r="259" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A259"/>
+      <c r="B259"/>
+      <c r="J259"/>
+      <c r="K259"/>
+      <c r="N259"/>
+    </row>
+    <row r="260" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A260"/>
+      <c r="B260"/>
+      <c r="J260"/>
+      <c r="K260"/>
+      <c r="N260"/>
+    </row>
+    <row r="261" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A261"/>
+      <c r="B261"/>
+      <c r="J261"/>
+      <c r="K261"/>
+      <c r="N261"/>
+    </row>
+    <row r="262" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A262"/>
+      <c r="B262"/>
+      <c r="J262"/>
+      <c r="K262"/>
+      <c r="N262"/>
+    </row>
+    <row r="263" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A263"/>
+      <c r="B263"/>
+      <c r="J263"/>
+      <c r="K263"/>
+      <c r="N263"/>
+    </row>
+    <row r="264" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A264"/>
+      <c r="B264"/>
+      <c r="J264"/>
+      <c r="K264"/>
+      <c r="N264"/>
+    </row>
+    <row r="265" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A265"/>
+      <c r="B265"/>
+      <c r="J265"/>
+      <c r="K265"/>
+      <c r="N265"/>
+    </row>
+    <row r="266" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A266"/>
+      <c r="B266"/>
+      <c r="J266"/>
+      <c r="K266"/>
+      <c r="N266"/>
+    </row>
+    <row r="267" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A267"/>
+      <c r="B267"/>
+      <c r="J267"/>
+      <c r="K267"/>
+      <c r="N267"/>
+    </row>
+    <row r="268" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A268"/>
+      <c r="B268"/>
+      <c r="J268"/>
+      <c r="K268"/>
+      <c r="N268"/>
+    </row>
+    <row r="269" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A269"/>
+      <c r="B269"/>
+      <c r="J269"/>
+      <c r="K269"/>
+      <c r="N269"/>
+    </row>
+    <row r="270" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A270"/>
+      <c r="B270"/>
+      <c r="J270"/>
+      <c r="K270"/>
+      <c r="N270"/>
+    </row>
+    <row r="271" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A271"/>
+      <c r="B271"/>
+      <c r="J271"/>
+      <c r="K271"/>
+      <c r="N271"/>
+    </row>
+    <row r="272" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A272"/>
+      <c r="B272"/>
+      <c r="J272"/>
+      <c r="K272"/>
+      <c r="N272"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:T67" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>